<commit_message>
Upgrade the wesite with visual and backend component
</commit_message>
<xml_diff>
--- a/server/data/Event_Registrations.xlsx
+++ b/server/data/Event_Registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -459,9 +459,29 @@
         <v>29/12/2025, 10:24:35 am</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Morning Zumba Blast</v>
+      </c>
+      <c r="C4" t="str">
+        <v>SWAPNIL HANUMANT LOKARE</v>
+      </c>
+      <c r="D4" t="str">
+        <v>sahilsingh3923@gmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>08788609431</v>
+      </c>
+      <c r="F4" t="str">
+        <v>7/4/2026, 11:58:58 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>